<commit_message>
Split contacts add into 4 type-specific subcommands
- Replace generic `wbox contacts add [type]` with dedicated subcommands:
  `add person`, `add household`, `add org`, `add trust`
- `add person` exposes person-specific flags: --prefix, --suffix,
  --nickname, --gender, --marital-status, --birth-date, --anniversary
- Household/Org/Trust require --name; Org/Trust share a private helper
  to avoid duplicating identical bodies
- Each subcommand gets --more-fields (JSON merge with reserved-key guard)
- Fix background_info → background_information in model and example file
- Use parse_more_fields utility in tasks.py instead of inlined equivalent

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resources/Contact Fields.xlsx
+++ b/resources/Contact Fields.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kadinb\Downloads\Code Projects\wealthbox-cli\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48245545-E3D5-493A-A55B-6A10FDC60529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63E8CA71-28FB-43A9-985B-85227B2AD104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6AD32C8B-08B2-4D2A-9FA0-FD304615E292}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="658" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="130">
   <si>
     <t>Person</t>
   </si>
@@ -360,9 +360,6 @@
   </si>
   <si>
     <t>While can be cleared by Empty String or None - will only ever show as empty string in returned objects. BUG - When doing an update from having a value to null, status code is 200 but the returned object will still contain the before value, but it will have succeeded, subsequent calls will confirm the date is removed.</t>
-  </si>
-  <si>
-    <t>SECURITY VULNERABILITY - Can assign any id with success, full name visible on web app</t>
   </si>
   <si>
     <t>Trying to remove using None or empty string fail silently, but it actually accepts the invalid entry and will display it on the web app. However when using the edit screen, it is rejected and the drop down just moves to the default "Select…"</t>
@@ -500,34 +497,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -939,13 +909,13 @@
         <v>90</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -968,7 +938,7 @@
         <v>90</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>97</v>
@@ -1026,7 +996,7 @@
         <v>98</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -1138,7 +1108,7 @@
         <v>105</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
@@ -1247,10 +1217,10 @@
         <v>90</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -1330,7 +1300,7 @@
         <v>89</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -1356,7 +1326,7 @@
         <v>101</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1382,7 +1352,7 @@
         <v>101</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1404,9 +1374,6 @@
       <c r="F23" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G23" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H23" s="2" t="s">
         <v>101</v>
       </c>
@@ -1430,9 +1397,6 @@
       <c r="F24" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G24" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H24" s="2" t="s">
         <v>101</v>
       </c>
@@ -1457,13 +1421,13 @@
         <v>90</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H25" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -1485,9 +1449,6 @@
       <c r="F26" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H26" s="2" t="s">
         <v>101</v>
       </c>
@@ -1515,7 +1476,7 @@
         <v>101</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
@@ -1537,9 +1498,6 @@
       <c r="F28" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G28" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H28" s="2" t="s">
         <v>101</v>
       </c>
@@ -1563,9 +1521,6 @@
       <c r="F29" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H29" s="2" t="s">
         <v>101</v>
       </c>
@@ -1610,13 +1565,13 @@
         <v>90</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H31" s="2" t="s">
         <v>101</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -1636,13 +1591,13 @@
         <v>90</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H32" s="2" t="s">
         <v>101</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
@@ -1662,7 +1617,7 @@
         <v>90</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
@@ -1682,7 +1637,7 @@
         <v>90</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -1708,7 +1663,7 @@
         <v>101</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1730,9 +1685,6 @@
       <c r="F36" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G36" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H36" s="2" t="s">
         <v>101</v>
       </c>
@@ -1757,13 +1709,13 @@
         <v>90</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -1789,7 +1741,7 @@
         <v>101</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -1812,13 +1764,13 @@
         <v>90</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H39" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
@@ -1841,7 +1793,7 @@
         <v>90</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H40" s="2" t="s">
         <v>101</v>
@@ -1866,9 +1818,6 @@
       <c r="F41" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G41" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H41" s="2" t="s">
         <v>101</v>
       </c>
@@ -1899,7 +1848,7 @@
         <v>101</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.25">
@@ -1922,7 +1871,7 @@
         <v>90</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H43" s="2" t="s">
         <v>101</v>
@@ -1948,7 +1897,7 @@
         <v>90</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H44" s="2" t="s">
         <v>101</v>
@@ -1974,7 +1923,7 @@
         <v>90</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H45" s="2" t="s">
         <v>101</v>
@@ -2003,7 +1952,7 @@
         <v>101</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
@@ -2026,13 +1975,13 @@
         <v>90</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H47" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
@@ -2058,7 +2007,7 @@
         <v>105</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
@@ -2084,7 +2033,7 @@
         <v>101</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
@@ -2107,13 +2056,13 @@
         <v>90</v>
       </c>
       <c r="G50" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="I50" s="2" t="s">
         <v>123</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
@@ -2135,9 +2084,6 @@
       <c r="F51" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G51" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H51" s="2" t="s">
         <v>101</v>
       </c>
@@ -2165,7 +2111,7 @@
         <v>105</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
@@ -2191,7 +2137,7 @@
         <v>105</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
@@ -2214,13 +2160,13 @@
         <v>90</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H54" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
@@ -2243,13 +2189,13 @@
         <v>90</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H55" s="2" t="s">
         <v>105</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
@@ -2295,7 +2241,7 @@
         <v>90</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H57" s="2" t="s">
         <v>101</v>
@@ -2347,7 +2293,7 @@
         <v>90</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H59" s="2" t="s">
         <v>101</v>
@@ -2373,7 +2319,7 @@
         <v>90</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H60" s="2" t="s">
         <v>101</v>
@@ -2399,7 +2345,7 @@
         <v>90</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H61" s="2" t="s">
         <v>101</v>
@@ -2428,7 +2374,7 @@
         <v>105</v>
       </c>
       <c r="I62" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
@@ -2451,7 +2397,7 @@
         <v>90</v>
       </c>
       <c r="H63" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
@@ -2477,7 +2423,7 @@
         <v>101</v>
       </c>
       <c r="I64" s="2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
@@ -2503,7 +2449,7 @@
         <v>101</v>
       </c>
       <c r="I65" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.25">
@@ -2532,7 +2478,7 @@
         <v>105</v>
       </c>
       <c r="I66" s="2" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.25">
@@ -2554,9 +2500,6 @@
       <c r="F67" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="G67" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H67" s="2" t="s">
         <v>101</v>
       </c>
@@ -2581,7 +2524,7 @@
         <v>90</v>
       </c>
       <c r="H68" s="2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.25">
@@ -2630,7 +2573,7 @@
         <v>89</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>101</v>
@@ -2760,7 +2703,7 @@
         <v>89</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H75" s="2" t="s">
         <v>98</v>
@@ -2858,13 +2801,13 @@
         <v>89</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H79" s="2" t="s">
         <v>98</v>
       </c>
       <c r="I79" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
@@ -2955,9 +2898,6 @@
       <c r="F83" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="G83" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="H83" s="2" t="s">
         <v>101</v>
       </c>
@@ -3025,7 +2965,7 @@
         <v>89</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>